<commit_message>
Normalize imported IC brief artifact references
</commit_message>
<xml_diff>
--- a/theos-past-research/outputs/workbooks/ABNB_edge_guidance_stock_reaction.xlsx
+++ b/theos-past-research/outputs/workbooks/ABNB_edge_guidance_stock_reaction.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4e854e651fda4841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guidance Events" sheetId="2" r:id="Rd8816299b0054dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Reactions" sheetId="3" r:id="R2672f49301434bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edge Observations" sheetId="4" r:id="R2fc25a688e054f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Bridge" sheetId="5" r:id="Ref01e96b94264c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OSE Trend" sheetId="6" r:id="R3be0dc209dfc425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="7" r:id="R0a0d4a6cfddd4c79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R8267fdbd16064175"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R42bf9f20d9fa4758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Reead8f60aff1413b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guidance Events" sheetId="2" r:id="Rd5e1fed1cdb74404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Reactions" sheetId="3" r:id="R04b8d95f814a472a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edge Observations" sheetId="4" r:id="R2c11b1d290e84701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Bridge" sheetId="5" r:id="Rc1624f589d954c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OSE Trend" sheetId="6" r:id="R814614874d484df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="7" r:id="R091bcb24b7f040a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R1382bb879557475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R16baec8e3ca14992"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -599,7 +599,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -609,7 +609,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -619,7 +619,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -629,7 +629,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -639,7 +639,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -649,7 +649,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -659,7 +659,7 @@
         <x:color rgb="FF17365D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF2F8"/>
         </x:patternFill>
       </x:fill>
@@ -669,7 +669,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -679,7 +679,7 @@
         <x:color rgb="FF17365D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF2F8"/>
         </x:patternFill>
       </x:fill>
@@ -689,7 +689,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -699,7 +699,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -709,7 +709,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -719,7 +719,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -730,7 +730,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -741,7 +741,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1243,7 +1243,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R27abf8e4727d41d2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca9dcda080df4a2c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1273,7 +1273,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R68d0d7e73a164c85"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R940e24d3b33742b6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1308,7 +1308,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra8d880a9bc5c4a58"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8cc715f04be6413f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3340,7 +3340,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38ba67994ebf4ef2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4dc0ab9f93d4094"/>
 </x:worksheet>
 </file>
 
@@ -4921,7 +4921,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fdf1b0060d848ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22378dd7c1f6480f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6811,7 +6811,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racc340812ab547ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re781f3edd1fb43ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11475,7 +11475,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88c6439ce9bb44d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R803e13659d23475d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11691,7 +11691,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7378a8c56c674ab3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6278c82b4911454d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12196,9 +12196,9 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cdb86273b2343f1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc439af649bf4092"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34974b699e04331"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7075b7fae1e454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40299,7 +40299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4655228039d40f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4a7a7b35b214c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40670,7 +40670,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R000f0ce63f264c8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69d660b5634749ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40878,7 +40878,7 @@
         <x:v>Point-in-time target panel</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>/Users/theomachado/Library/CloudStorage/OneDrive-UniversityofFlorida/CAIMANES/CITADEL 2026/research/readiness/20260903T053309Z_abnb_readiness/target_panel.csv</x:v>
+        <x:v>research/readiness/20260903T053309Z_abnb_readiness/target_panel.csv</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
         <x:v>As preserved in panel</x:v>
@@ -40907,7 +40907,7 @@
         <x:v>Transcript index</x:v>
       </x:c>
       <x:c r="E8" s="29" t="str">
-        <x:v>/Users/theomachado/Library/CloudStorage/OneDrive-UniversityofFlorida/CAIMANES/CITADEL 2026/research/transcripts/transcript_index.csv</x:v>
+        <x:v>research/transcripts/transcript_index.csv</x:v>
       </x:c>
       <x:c r="F8" s="19" t="str">
         <x:v>Indexed 2026-09-03</x:v>
@@ -40994,7 +40994,7 @@
         <x:v>Frozen hypotheses and minimum-evidence gates</x:v>
       </x:c>
       <x:c r="E11" s="29" t="str">
-        <x:v>/Users/theomachado/Library/CloudStorage/OneDrive-UniversityofFlorida/CAIMANES/CITADEL 2026/research/hypothesis_ledger.csv</x:v>
+        <x:v>research/hypothesis_ledger.csv</x:v>
       </x:c>
       <x:c r="F11" s="19" t="str">
         <x:v>2026-09-03</x:v>
@@ -41015,7 +41015,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcfdb0e0622b4bbf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3788a8aca80547ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>